<commit_message>
fix(dgii): calibrate row heights and merged cell layout in IST XLSX template to prevent clipping
</commit_message>
<xml_diff>
--- a/resources/templates/dgii/IST-Telecomunicaciones-253-12.xlsx
+++ b/resources/templates/dgii/IST-Telecomunicaciones-253-12.xlsx
@@ -710,7 +710,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="179">
+  <cellXfs count="180">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="2" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="true">
       <protection hidden="false"/>
     </xf>
@@ -1354,13 +1354,20 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
       <protection hidden="false"/>
     </xf>
-    <xf xfId="0" fontId="12" numFmtId="0" fillId="4" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="true">
-      <protection hidden="false"/>
-    </xf>
-    <xf xfId="0" fontId="13" numFmtId="0" fillId="4" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="true">
-      <protection hidden="false"/>
-    </xf>
-    <xf xfId="0" fontId="14" numFmtId="0" fillId="4" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="true">
+    <xf xfId="0" fontId="12" numFmtId="0" fillId="4" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="true">
+      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+      <protection hidden="false"/>
+    </xf>
+    <xf xfId="0" fontId="13" numFmtId="0" fillId="4" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="true">
+      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+      <protection hidden="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="4" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="true">
+      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+      <protection hidden="false"/>
+    </xf>
+    <xf xfId="0" fontId="14" numFmtId="0" fillId="4" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="true">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
       <protection hidden="false"/>
     </xf>
   </cellXfs>
@@ -1379,9 +1386,9 @@
       <xdr:col>1</xdr:col>
       <xdr:colOff>38100</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="523875" cy="514350"/>
+    <xdr:ext cx="466725" cy="457200"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="DGII_Logo" descr="Logo DGII"/>
@@ -1992,27 +1999,27 @@
       <c r="AD1" s="1"/>
       <c r="AE1" s="1"/>
     </row>
-    <row r="2" spans="1:257" customHeight="1" ht="12">
+    <row r="2" spans="1:257" customHeight="1" ht="16">
       <c r="A2" s="1"/>
       <c r="B2" s="3"/>
       <c r="D2" s="176" t="s">
         <v>67</v>
       </c>
-      <c r="Z2" s="178" t="s">
+      <c r="X2" s="179" t="s">
         <v>70</v>
       </c>
       <c r="AE2" s="1"/>
     </row>
-    <row r="3" spans="1:257" customHeight="1" ht="12">
+    <row r="3" spans="1:257" customHeight="1" ht="15">
       <c r="A3" s="1"/>
       <c r="D3" s="177" t="s">
         <v>68</v>
       </c>
       <c r="AE3" s="1"/>
     </row>
-    <row r="4" spans="1:257" customHeight="1" ht="12">
+    <row r="4" spans="1:257" customHeight="1" ht="14">
       <c r="A4" s="1"/>
-      <c r="D4" s="64" t="s">
+      <c r="D4" s="178" t="s">
         <v>69</v>
       </c>
       <c r="AE4" s="1"/>
@@ -3662,6 +3669,10 @@
     <mergeCell ref="D25:S25"/>
     <mergeCell ref="D26:S26"/>
     <mergeCell ref="D27:S27"/>
+    <mergeCell ref="D2:W2"/>
+    <mergeCell ref="D3:W3"/>
+    <mergeCell ref="D4:W4"/>
+    <mergeCell ref="X2:AC4"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="true"/>
   <pageMargins left="0.15748031496063" right="0.47244094488189" top="0.19685039370079" bottom="0.19685039370079" header="0.15748031496063" footer="0.23622047244094"/>

</xml_diff>